<commit_message>
feat: integrate GrabMart scrapers, purge unused tables, consolidate 3 Metabase dashboards, and update docs
</commit_message>
<xml_diff>
--- a/thesis/Literature_Review_Matrix.xlsx
+++ b/thesis/Literature_Review_Matrix.xlsx
@@ -13,10 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cambodia CPI Methodology" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Literature Review Matrix'!$A$1:$K$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Thematic Pillars &amp; Pipeline'!$A$1:$F$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Methodology &amp; Metrics Benchmark'!$A$1:$G$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Cambodia CPI Methodology'!$A$1:$G$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Literature Review Matrix'!$A$3:$K$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -25,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,24 +31,86 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Segoe UI"/>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <sz val="11"/>
+      <name val="Segoe UI"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002F5597"/>
+        <bgColor rgb="002F5597"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+        <bgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F5F9"/>
+        <bgColor rgb="00F2F5F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+        <bgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -59,26 +118,96 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00FFFFFF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00FFFFFF"/>
+      </right>
+      <top style="medium">
+        <color rgb="001F4E79"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="001F4E79"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -445,14 +574,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
     <col width="28" customWidth="1" min="6" max="6"/>
     <col width="35" customWidth="1" min="7" max="7"/>
     <col width="30" customWidth="1" min="8" max="8"/>
@@ -461,685 +590,713 @@
     <col width="30" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="40" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>CAMBODIA DAILY CPI MEDALLION PIPELINE — SYSTEMATIC LITERATURE REVIEW MATRIX</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Comprehensive Academic &amp; Institutional Literature Synthesis (Chapter II: Literature Review)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Pillar / Domain</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Study / Paper Title</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Study / Paper</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Authors</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>Journal / Publisher / Outlet</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Key Methodology &amp; Algorithms</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Dataset &amp; Experimental Scope</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Reported Metrics &amp; Empirical Results</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>Relevance &amp; Mapping to Cambodia CPI Pipeline</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>DOI / Citation Link</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="4" ht="70" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>LR-01</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>1. High-Frequency Web Scraping</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>The Billion Prices Project: Using Online Prices for Measurement and Research</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>Alberto Cavallo &amp; Roberto Rigobon</t>
         </is>
       </c>
-      <c r="E2" s="5" t="n">
+      <c r="E4" s="7" t="n">
         <v>2016</v>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>Journal of Economic Perspectives (Vol. 30, No. 2, pp. 151-178)</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>Automated daily web scrapers, Jevons geometric mean, high-frequency online micro price tracking.</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="H4" s="6" t="inlineStr">
         <is>
           <t>Hundreds of multi-channel &amp; pure e-commerce retailers across 22 countries; billions of individual price quotes.</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="I4" s="6" t="inlineStr">
         <is>
           <t>• Pearson correlation &gt;0.98 with official monthly CPI in low-inflation economies (US, Germany, Japan, Brazil).
 • Detected true 20.0% inflation in Argentina (2007–2015) vs 8.0% official reported rate.
 • Detected exchange rate pass-through shocks within 3–14 days (vs 30–60 days official lag).</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="J4" s="6" t="inlineStr">
         <is>
           <t>Provides empirical foundation for daily automated crawling of Cambodian retail e-commerce platforms to eliminate publication lag and capture rapid currency/pass-through shocks.</t>
         </is>
       </c>
-      <c r="K2" s="4" t="inlineStr">
+      <c r="K4" s="8" t="inlineStr">
         <is>
           <t>https://doi.org/10.1257/jep.30.2.151</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="5" ht="70" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>LR-02</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>1. High-Frequency Web Scraping</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>Web scraping techniques to collect data on consumer prices and machine learning for product classification</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D5" s="11" t="inlineStr">
         <is>
           <t>Federico Polidoro, Roberto Giannini, Rosanna Lo Conte, &amp; Silvia Rossetti</t>
         </is>
       </c>
-      <c r="E3" s="5" t="n">
+      <c r="E5" s="12" t="n">
         <v>2015</v>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F5" s="11" t="inlineStr">
         <is>
           <t>Statistical Journal of the IAOS (Vol. 31, No. 3, pp. 447-461)</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G5" s="11" t="inlineStr">
         <is>
           <t>Automated scraping architectures, HTML parsing pipelines, text preprocessing, Naive Bayes and Support Vector Machine (SVM) classification.</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H5" s="11" t="inlineStr">
         <is>
           <t>Italian National Institute of Statistics (ISTAT) empirical scanner &amp; web scraping pilot on consumer electronics and groceries.</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="I5" s="11" t="inlineStr">
         <is>
           <t>• Increased quote sample size by &gt;100x (over two orders of magnitude).
 • Reduced field collection labor costs by &gt;80%.
 • Classification accuracy ranged from 82% to 92.5% across product groups.</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="J5" s="11" t="inlineStr">
         <is>
           <t>Demonstrates the operational viability of substituting manual field enumerator surveys with automated web crawlers in official NSI production pipelines.</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="K5" s="13" t="inlineStr">
         <is>
           <t>https://doi.org/10.3233/SJI-150896</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="6" ht="70" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>LR-03</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>1. High-Frequency Web Scraping</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Practical Guide on the Use of Web Scraping for the Calculation of the Harmonised Index of Consumer Prices (HICP)</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>Eurostat (Statistical Office of the European Communities)</t>
         </is>
       </c>
-      <c r="E4" s="5" t="n">
+      <c r="E6" s="7" t="n">
         <v>2022</v>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>Eurostat Methodological Guidelines (Luxembourg)</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>Crawler rate-limiting, robot.txt compliance, anti-bot mitigation, missing quote handling, longitudinal product ID hashing.</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>Standardized institutional guidelines across 27 EU National Statistical Institutes.</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="I6" s="6" t="inlineStr">
         <is>
           <t>• Standardized crawler governance, ethical scraping protocols, and data protection.
 • Codified 7-day price carry-forward and geometric imputation rules for missing scraped quotes.</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="J6" s="6" t="inlineStr">
         <is>
           <t>Directly guides the Bronze ingestion layer design, respecting robot policies, retry-backoff algorithms, and raw payload data lake storage.</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr">
+      <c r="K6" s="6" t="inlineStr">
         <is>
           <t>Eurostat Practical Guide (2022)</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="7" ht="70" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>LR-04</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>2. NLP &amp; AI in Product Classification</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr">
         <is>
           <t>NLP-Enhanced Inflation Measurement Using BERT and Web Scraping</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D7" s="11" t="inlineStr">
         <is>
           <t>Martin Berki, Vanesa Andicsova, &amp; Milos Oravec</t>
         </is>
       </c>
-      <c r="E5" s="5" t="n">
+      <c r="E7" s="12" t="n">
         <v>2025</v>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F7" s="11" t="inlineStr">
         <is>
           <t>Frontiers in Artificial Intelligence (Vol. 8, Art. 1543026)</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G7" s="11" t="inlineStr">
         <is>
           <t>Fine-tuned BERT transformer architecture for multi-class hierarchical text classification into 5-digit COICOP codes.</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H7" s="11" t="inlineStr">
         <is>
           <t>Over 100,000 scraped e-commerce product titles across retail supermarkets.</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="I7" s="11" t="inlineStr">
         <is>
           <t>• Overall classification accuracy: 94.56%.
 • Weighted precision: 94.07%.
 • Outperformed rule-based regex and TF-IDF baselines on noisy, abbreviated product listings.</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="J7" s="11" t="inlineStr">
         <is>
           <t>Forms the technical foundation for the Silver classification layer, validating transformer embeddings for classifying Cambodian e-commerce items into 12 COICOP divisions.</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="K7" s="13" t="inlineStr">
         <is>
           <t>https://doi.org/10.3389/frai.2025.1543026</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="8" ht="70" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>LR-05</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>2. NLP &amp; AI in Product Classification</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>Project Spectrum: Using Generative AI to Enhance Inflation Nowcasting</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>Bank for International Settlements (BIS), European Central Bank (ECB), &amp; Deutsche Bundesbank</t>
         </is>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="E8" s="7" t="n">
         <v>2024</v>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>BIS Innovation Hub Technical Report (Basel, Switzerland)</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>Large Language Models (LLMs), dense vector embeddings, vector database caching, few-shot prompt engineering.</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Large Language Models (LLMs), dense vector embeddings (OpenAI / Cohere), vector database caching, few-shot prompt engineering.</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>Billions of scraped price quotes across multi-lingual European retailer catalogs.</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="I8" s="6" t="inlineStr">
         <is>
           <t>• Zero-shot &amp; few-shot LLM reasoning achieved &gt;95% classification precision.
 • Reduced batch processing latency from several days to &lt;3 minutes via vector memoization and cache lookup.</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="J8" s="6" t="inlineStr">
         <is>
           <t>Validates the hybrid Silver layer architecture: using dense vector caching for instant exact match and LLM fallback for ambiguous Khmer/English product descriptions.</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="K8" s="8" t="inlineStr">
         <is>
           <t>https://www.bis.org/about/bisih/topics/ai/spectrum.htm</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="9" ht="70" customHeight="1">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>LR-06</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>2. NLP &amp; AI in Product Classification</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C9" s="11" t="inlineStr">
         <is>
           <t>Using Machine Learning for Classifying Web-Scraped Data into COICOP</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D9" s="11" t="inlineStr">
         <is>
           <t>Office for National Statistics (ONS) Data Science Campus</t>
         </is>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E9" s="12" t="n">
         <v>2020</v>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F9" s="11" t="inlineStr">
         <is>
           <t>ONS Methodology Technical Paper (Newport, UK)</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G9" s="11" t="inlineStr">
         <is>
           <t>FastText &amp; TF-IDF feature extraction, XGBoost classifier, Human-in-the-Loop (HITL) operational confidence thresholding.</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="H9" s="11" t="inlineStr">
         <is>
           <t>UK web-scraped clothing and grocery price panel (millions of quotes).</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="I9" s="11" t="inlineStr">
         <is>
           <t>• Macro F1-score of 87%–91%.
 • Confidence threshold (tau = 0.80) allowed &gt;70% of volume to be fully automated without human intervention while maintaining official statistical quality.</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr">
+      <c r="J9" s="11" t="inlineStr">
         <is>
           <t>Informs the automated Silver validation pipeline: items with classification confidence &gt;= 0.80 pass automatically, while low-confidence items are flagged for audit.</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr">
+      <c r="K9" s="13" t="inlineStr">
         <is>
           <t>https://www.ons.gov.uk/economy/inflationandpriceindices/methodologies</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="10" ht="70" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>LR-07</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>3. Econometric Index Number Theory</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Consumer Price Index Manual: Concepts and Methods</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>IMF, ILO, OECD, Eurostat, UN, &amp; World Bank</t>
         </is>
       </c>
-      <c r="E8" s="5" t="n">
+      <c r="E10" s="7" t="n">
         <v>2020</v>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>International Monetary Fund (Washington, D.C.)</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>Axiomatic price index theory, elementary Jevons geometric mean, Carli/Dutot formula bias proofs, missing quote imputation, hedonic quality adjustment.</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>Global standard methodology for national statistical offices and central banks.</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="I10" s="6" t="inlineStr">
         <is>
           <t>• Proved Jevons geometric mean satisfies time-reversal and transitivity axioms.
 • Proved Carli arithmetic mean suffers from 0.5%–1.5% upward price bounce bias.
 • Mandated Jevons formula as the global best practice for unweighted micro-level aggregation.</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr">
+      <c r="J10" s="6" t="inlineStr">
         <is>
           <t>Governs the Gold aggregation layer: proves why elementary daily micro-indices in the pipeline must use Jevons geometric averages rather than arithmetic means.</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr">
+      <c r="K10" s="6" t="inlineStr">
         <is>
           <t>ISBN: 978-1-48435-430-8</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="11" ht="70" customHeight="1">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>LR-08</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>3. Econometric Index Number Theory</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C11" s="11" t="inlineStr">
         <is>
           <t>Substitution Bias and Scanner Data: Measuring Price Change with Scanner Data</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D11" s="11" t="inlineStr">
         <is>
           <t>W. Erwin Diewert &amp; Kevin J. Fox</t>
         </is>
       </c>
-      <c r="E9" s="5" t="n">
+      <c r="E11" s="12" t="n">
         <v>2020</v>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F11" s="11" t="inlineStr">
         <is>
           <t>Journal of Econometrics (Vol. 217, No. 2, pp. 268-284)</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="G11" s="11" t="inlineStr">
         <is>
           <t>Superlative index number formulas (Fisher Ideal, Törnqvist), exact economic index theory, second-order Taylor approximations.</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="H11" s="11" t="inlineStr">
         <is>
           <t>High-frequency barcode scanner transactions across extensive supermarket chains.</t>
         </is>
       </c>
-      <c r="I9" s="4" t="inlineStr">
+      <c r="I11" s="11" t="inlineStr">
         <is>
           <t>• Quantified that standard fixed-basket Laspeyres indices overstate inflation by 0.30%–0.85% per annum due to commodity substitution.
 • Proved superlative indices effectively eliminate substitution bias by capturing shifts toward discounted goods.</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr">
+      <c r="J11" s="11" t="inlineStr">
         <is>
           <t>Justifies the pipeline's hybrid weighting strategy, combining official CSES fixed weights with dynamic expenditure approximations.</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr">
+      <c r="K11" s="13" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.jeconom.2019.12.013</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="12" ht="70" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>LR-09</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>3. Econometric Index Number Theory</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>A New Methodology for Processing Scanner Data in the Dutch CPI</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>Antonio G. Chessa</t>
         </is>
       </c>
-      <c r="E10" s="5" t="n">
+      <c r="E12" s="7" t="n">
         <v>2016</v>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>EURONA — Eurostat Review on National Accounts (Vol. 2016, No. 1, pp. 49-69)</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>Rolling Multilateral GEKS-Törnqvist index, Quality-Adjusted Unit Value GEKS (QU-GEKS), Movement Splice / Window Splicing (13-month rolling window).</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>Statistics Netherlands (CBS) comprehensive supermarket scanner data panel.</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr">
+      <c r="I12" s="6" t="inlineStr">
         <is>
           <t>• Proved multilateral GEKS completely eliminates 'chain drift' (5%–10% cumulative multi-year bias caused by clearance sales and item turnover).
 • Successfully deployed into official Dutch national CPI production.</t>
         </is>
       </c>
-      <c r="J10" s="4" t="inlineStr">
+      <c r="J12" s="6" t="inlineStr">
         <is>
           <t>Provides the theoretical framework for multilateral aggregation in the Gold layer to prevent downward chain drift caused by frequent flash sales on Cambodian e-commerce platforms.</t>
         </is>
       </c>
-      <c r="K10" s="4" t="inlineStr">
+      <c r="K12" s="6" t="inlineStr">
         <is>
           <t>EURONA 2016(1):49-69</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="13" ht="70" customHeight="1">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>LR-10</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>4. ML &amp; Time-Series Nowcasting</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C13" s="11" t="inlineStr">
         <is>
           <t>Nowcasting Food Inflation with a Massive Amount of Online Prices</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D13" s="11" t="inlineStr">
         <is>
           <t>Pawel Macias, Damian Stelmasiak, &amp; Karol Szafranek</t>
         </is>
       </c>
-      <c r="E11" s="5" t="n">
+      <c r="E13" s="12" t="n">
         <v>2023</v>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F13" s="11" t="inlineStr">
         <is>
           <t>International Journal of Forecasting (Vol. 39, No. 2, pp. 809-826)</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="G13" s="11" t="inlineStr">
         <is>
           <t>Mixed-Data Sampling (MIDAS), Autoregressive Distributed Lag (ARDL), daily scraped web panel aggregation for monthly macroeconomic forecasting.</t>
         </is>
       </c>
-      <c r="H11" s="4" t="inlineStr">
+      <c r="H13" s="11" t="inlineStr">
         <is>
           <t>Over 2 million daily food quotes scraped over an 11-year longitudinal panel in Poland.</t>
         </is>
       </c>
-      <c r="I11" s="4" t="inlineStr">
+      <c r="I13" s="11" t="inlineStr">
         <is>
           <t>• 15% to 35% reduction in Root Mean Square Error (RMSE) over standard AR/ARIMA benchmarks when predicting official monthly food CPI.
 • Superior real-time tracking during periods of high economic turbulence and supply shocks.</t>
         </is>
       </c>
-      <c r="J11" s="4" t="inlineStr">
+      <c r="J13" s="11" t="inlineStr">
         <is>
           <t>Directly validates the Gold-to-Platinum nowcasting module: using daily scraped food &amp; beverage sub-indices to nowcast official National Institute of Statistics (NIS) monthly inflation.</t>
         </is>
       </c>
-      <c r="K11" s="4" t="inlineStr">
+      <c r="K13" s="13" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.ijforecast.2022.01.007</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="14" ht="70" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>LR-11</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>4. ML &amp; Time-Series Nowcasting</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>Forecasting Inflation in a Data-Rich Environment: The Benefits of Machine Learning Methods</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>Marcelo C. Medeiros, Gabriel F. R. Vasconcelos, Alvaro Veiga, &amp; Eduardo Zilberman</t>
         </is>
       </c>
-      <c r="E12" s="5" t="n">
+      <c r="E14" s="7" t="n">
         <v>2021</v>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>Journal of Business &amp; Economic Statistics (Vol. 39, No. 1, pp. 98-119)</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>Random Forests, Gradient Boosted Regression Trees (GBRT/LightGBM), LASSO, Ridge, Factor Models vs. Phillips Curve and AR benchmarks.</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="H14" s="6" t="inlineStr">
         <is>
           <t>Extensive high-dimensional US macroeconomic dataset (FRED-MD) across 1 to 12-month forecast horizons.</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr">
+      <c r="I14" s="6" t="inlineStr">
         <is>
           <t>• Tree-based ensembles (Random Forest &amp; GBRT) significantly outperformed all linear econometric benchmarks, reducing MSFE by 10%–25%.
 • Effectively captured non-linear threshold effects and complex macro interactions between commodities, exchange rates, and prices.</t>
         </is>
       </c>
-      <c r="J12" s="4" t="inlineStr">
+      <c r="J14" s="6" t="inlineStr">
         <is>
           <t>Informs the pipeline's multi-horizon forecasting engine, supporting gradient boosting ensembles with commodity and KHR/USD exchange rate regressors.</t>
         </is>
       </c>
-      <c r="K12" s="4" t="inlineStr">
+      <c r="K14" s="8" t="inlineStr">
         <is>
           <t>https://doi.org/10.1080/07350015.2019.1637745</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K12"/>
+  <autoFilter ref="A3:K14"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A1:K1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId8"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1150,7 +1307,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1161,57 +1318,64 @@
     <col width="45" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="40" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>THEMATIC RESEARCH PILLARS &amp; MEDALLION ARCHITECTURE MAPPING</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
           <t>Pillar #</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Thematic Research Domain</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Core Academic &amp; Institutional Literature</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Key Methodological Principles</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>Target Medallion Layer</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>Engineering Implementation in Cambodia Pipeline</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="4" ht="95" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Pillar 1</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>High-Frequency Web Scraping &amp; Ingestion</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>• Cavallo &amp; Rigobon (2016) [BPP]
 • Polidoro et al. (2015) [ISTAT]
 • Eurostat (2022) [HICP Guide]</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>• Automated daily distributed crawlers.
 • &gt;100x sample size expansion over manual surveys.
@@ -1219,36 +1383,36 @@
 • 7-day missing price carry-forward rules.</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E4" s="14" t="inlineStr">
         <is>
           <t>Bronze Layer (Raw Ingestion)</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>Daily Playwright/HTTP crawlers targeting 19 Cambodian retail/telecom/transport/hotel sources + MEF FX storing raw JSON/HTML payloads in PostgreSQL bronze.raw_prices and staging.raw_scrapes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Daily Playwright/Scrapy crawlers targeting major Cambodian supermarkets (AEON, Chip Mong, Makro, Nham24) storing raw JSON/HTML payloads in PostgreSQL / Data Lake.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="95" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>Pillar 2</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>NLP &amp; AI in Product Classification</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>• Berki et al. (2025) [BERT COICOP]
 • BIS / ECB / Bundesbank (2024) [Spectrum]
 • ONS Data Science Campus (2020) [XGBoost]</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D5" s="11" t="inlineStr">
         <is>
           <t>• Dense transformer embeddings (BERT/RoBERTa).
 • Multi-class hierarchical classification into 12 COICOP divisions.
@@ -1256,90 +1420,92 @@
 • Human-in-the-Loop (HITL) thresholding (tau &gt;= 0.80).</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E5" s="15" t="inlineStr">
         <is>
           <t>Silver Layer (Enrichment &amp; Standardization)</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Hybrid text processing: 15 pure store domain locks + 12-division reference vector cosine matching + Gemini Pro/Flash AI fallback cached in silver.dim_coicop_ai_cache.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>Hybrid text processing: vector embedding semantic search against COICOP codebook + LLM fallback for multi-lingual (Khmer/English) listings with confidence auditing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="95" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Pillar 3</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Econometric Multilateral Index Theory</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>• IMF/ILO/UN CPI Manual (2020)
 • Diewert &amp; Fox (2020) [Substitution Bias]
 • Chessa (2016) [GEKS / Statistics Netherlands]</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>• Unweighted Jevons geometric mean satisfies time-reversal &amp; transitivity.
 • Superlative Fisher/Törnqvist eliminates substitution bias (0.3%–0.85%/yr).
-• ILO class-mean imputation advances prices for missing items.</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
+• Rolling Multilateral GEKS with movement splice eliminates chain drift.</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>Gold Layer (Aggregations &amp; Analytics)</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>Two-stage aggregation: Jevons geometric mean for elementary item price ratios (gold.fct_elementary_indices) + Laspeyres fixed-weight division roll-up into headline/core CPI (gold.fct_cpi_daily).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>dbt transformation models executing elementary Jevons daily indexing, aggregation into 12 COICOP groups, and multilateral GEKS adjustments for product turnover.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="95" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>Pillar 4</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>Machine Learning &amp; Macro Nowcasting</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr">
         <is>
           <t>• Macias et al. (2023) [MIDAS Nowcasting]
 • Medeiros et al. (2021) [ML Inflation]</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D7" s="11" t="inlineStr">
         <is>
           <t>• Mixed-Data Sampling (MIDAS) bridging daily online prices to monthly official CPI.
 • 15%–35% RMSE reduction over AR/ARIMA.
 • Gradient Boosted Trees (GBRT/LightGBM) &amp; Random Forests capturing non-linear macro interactions.</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E7" s="15" t="inlineStr">
         <is>
           <t>Platinum Layer (Nowcasting &amp; Dashboards)</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F7" s="11" t="inlineStr">
         <is>
           <t>Ensemble forecasting models predicting official National Institute of Statistics (NIS) monthly CPI 20–30 days prior to official publication using daily scraped indexes + exchange rates.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F5"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1350,7 +1516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1362,341 +1528,350 @@
     <col width="22" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="40" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>METHODOLOGICAL BENCHMARK &amp; METRIC TAXONOMY</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Algorithm / Formula</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Benchmark / Baseline</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Key Metric / Reported Performance</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>Advantages</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>Limitations / Tradeoffs</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Reference Paper</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="4" ht="65" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>NLP Classification</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>BERT Transformer (Fine-Tuned)</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>TF-IDF + Naive Bayes / SVM</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>94.56% Accuracy, 94.07% Precision</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>Deep contextual semantic understanding; handles abbreviations, brands, packaging nuances.</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>Higher computational footprint; requires GPU or inference optimization.</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>Berki et al. (2025)</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="5" ht="65" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>NLP Classification</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>LLM + Vector Cache (Project Spectrum)</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>Handcrafted Regex Rules</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D5" s="10" t="inlineStr">
         <is>
           <t>&gt;95% Precision, Latency &lt;3 min</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E5" s="11" t="inlineStr">
         <is>
           <t>Zero-shot/few-shot multi-lingual adaptation (Khmer/English); fast retrieval via caching.</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F5" s="11" t="inlineStr">
         <is>
           <t>API token costs; potential non-deterministic hallucinations if unconstrained.</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G5" s="11" t="inlineStr">
         <is>
           <t>BIS / ECB / Bundesbank (2024)</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="6" ht="65" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>NLP Classification</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>FastText + XGBoost with HITL (tau=0.80)</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Manual Field Survey Categorization</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>87%–91% Macro F1, &gt;70% Automated</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>Lightweight, deterministic confidence scores; high throughput for automated pipelines.</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>Slightly lower accuracy on rare out-of-vocabulary product items.</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>ONS Data Science Campus (2020)</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="7" ht="65" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>Index Calculation</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>Jevons Geometric Mean</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr">
         <is>
           <t>Carli Arithmetic Mean / Dutot Ratio</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D7" s="10" t="inlineStr">
         <is>
           <t>Eliminates 0.5%–1.5% Upward Bias</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E7" s="11" t="inlineStr">
         <is>
           <t>Axiomatically sound (satisfies time-reversal &amp; transitivity); standard for unweighted micro prices.</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F7" s="11" t="inlineStr">
         <is>
           <t>Cannot handle zero prices without imputation or shift constants.</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G7" s="11" t="inlineStr">
         <is>
           <t>IMF CPI Manual (2020)</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="8" ht="65" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Index Calculation</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Superlative Indices (Fisher / Törnqvist)</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>Fixed-base Laspeyres Index</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>Removes 0.3%–0.85%/yr Substitution Bias</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>Exact second-order approximation to true cost of living; accommodates consumer substitution.</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>Requires simultaneous real-time quantity/expenditure weights.</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>Diewert &amp; Fox (2020)</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="9" ht="65" customHeight="1">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>Index Calculation</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>Rolling Multilateral GEKS (Movement Splice)</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C9" s="11" t="inlineStr">
         <is>
           <t>Direct Bilateral Chained Indices</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D9" s="10" t="inlineStr">
         <is>
           <t>Eliminates 5%–10% Cumulative Chain Drift</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E9" s="11" t="inlineStr">
         <is>
           <t>Prevents multi-year downward/upward drift caused by clearance sales and item turnover.</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F9" s="11" t="inlineStr">
         <is>
           <t>Requires rolling multi-month observation window (e.g. 13 months).</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G9" s="11" t="inlineStr">
         <is>
           <t>Chessa / CBS (2016)</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="10" ht="65" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Time-Series Nowcasting</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>MIDAS Regression (Mixed-Data Sampling)</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Traditional AR / ARIMA</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>15%–35% RMSE Reduction</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>Directly integrates high-frequency daily scraped data into monthly target forecasts without aggregation loss.</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>Linear parameterization assumptions.</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>Macias et al. (2023)</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="11" ht="65" customHeight="1">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>Time-Series Nowcasting</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>Gradient Boosted Trees (GBRT / LightGBM)</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C11" s="11" t="inlineStr">
         <is>
           <t>Phillips Curve / Factor Models</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D11" s="10" t="inlineStr">
         <is>
           <t>10%–25% MSFE Reduction</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E11" s="11" t="inlineStr">
         <is>
           <t>Captures non-linearities, threshold effects, and commodity/exchange rate shocks without overfitting.</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F11" s="11" t="inlineStr">
         <is>
           <t>Black-box nature requires SHAP/feature importance for economic interpretability.</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="G11" s="11" t="inlineStr">
         <is>
           <t>Medeiros et al. (2021)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G9"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1707,7 +1882,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1719,526 +1894,543 @@
     <col width="35" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="40" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>OFFICIAL CAMBODIA CPI METHODOLOGY &amp; EXPENDITURE BASKET (NIS / IMF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Two-Stage Aggregation: Jevons Geometric Mean (Elementary Items) + Modified Laspeyres (12 COICOP Divisions)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
           <t>COICOP Div</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Division Name (UN Standard)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Official Weight (%)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Elementary Aggregation Method</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>Division Aggregation Method</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>Economic Rationale &amp; Sensitivity</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Official Authority &amp; Survey Basis</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="4" ht="40" customHeight="1">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>01</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Food and Non-Alcoholic Beverages</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C4" s="16" t="inlineStr">
         <is>
           <t>44.800%</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D4" s="16" t="inlineStr">
         <is>
           <t>Jevons Geometric Mean</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E4" s="16" t="inlineStr">
         <is>
           <t>Modified Laspeyres</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>Largest expenditure share (~45%); extreme sensitivity to agricultural supply &amp; weather.</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>NIS Cambodia / CSES Household Survey</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="5" ht="40" customHeight="1">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>02</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>Alcoholic Beverages, Tobacco &amp; Narcotics</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C5" s="17" t="inlineStr">
         <is>
           <t>1.500%</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D5" s="17" t="inlineStr">
         <is>
           <t>Jevons Geometric Mean</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E5" s="17" t="inlineStr">
         <is>
           <t>Modified Laspeyres</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F5" s="11" t="inlineStr">
         <is>
           <t>Excise tax driven, inelastic consumption patterns.</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G5" s="11" t="inlineStr">
         <is>
           <t>NIS Cambodia / CSES Household Survey</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>03</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Clothing and Footwear</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C6" s="16" t="inlineStr">
         <is>
           <t>2.900%</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D6" s="16" t="inlineStr">
         <is>
           <t>Jevons Geometric Mean</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E6" s="16" t="inlineStr">
         <is>
           <t>Modified Laspeyres</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>Subject to seasonal discounting and apparel churn.</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>NIS Cambodia / CSES Household Survey</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>04</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Housing, Water, Electricity, Gas &amp; Fuels</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C7" s="17" t="inlineStr">
         <is>
           <t>17.100%</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D7" s="17" t="inlineStr">
         <is>
           <t>Jevons Geometric Mean</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E7" s="17" t="inlineStr">
         <is>
           <t>Modified Laspeyres</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F7" s="11" t="inlineStr">
         <is>
           <t>Second largest share (~17%); utility tariffs (EDC/PPWSA) &amp; cooking gas.</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G7" s="11" t="inlineStr">
         <is>
           <t>NIS Cambodia / CSES Household Survey</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>05</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Furnishings &amp; Routine Household Maintenance</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C8" s="16" t="inlineStr">
         <is>
           <t>3.300%</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D8" s="16" t="inlineStr">
         <is>
           <t>Jevons Geometric Mean</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E8" s="16" t="inlineStr">
         <is>
           <t>Modified Laspeyres</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>Durable goods, household detergents, appliances.</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>NIS Cambodia / CSES Household Survey</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="9" ht="40" customHeight="1">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>06</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>Health</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C9" s="17" t="inlineStr">
         <is>
           <t>5.600%</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D9" s="17" t="inlineStr">
         <is>
           <t>Jevons Geometric Mean</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E9" s="17" t="inlineStr">
         <is>
           <t>Modified Laspeyres</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F9" s="11" t="inlineStr">
         <is>
           <t>Pharmaceuticals and healthcare clinic expenditures.</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G9" s="11" t="inlineStr">
         <is>
           <t>NIS Cambodia / CSES Household Survey</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="10" ht="40" customHeight="1">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>07</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Transport</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C10" s="16" t="inlineStr">
         <is>
           <t>12.200%</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D10" s="16" t="inlineStr">
         <is>
           <t>Jevons Geometric Mean</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E10" s="16" t="inlineStr">
         <is>
           <t>Modified Laspeyres</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>Third largest share (~12%); direct passthrough from global oil &amp; MOC fuel prices.</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>NIS Cambodia / CSES Household Survey</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="11" ht="40" customHeight="1">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>08</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>Communication</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C11" s="17" t="inlineStr">
         <is>
           <t>3.900%</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D11" s="17" t="inlineStr">
         <is>
           <t>Jevons Geometric Mean</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E11" s="17" t="inlineStr">
         <is>
           <t>Modified Laspeyres</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F11" s="11" t="inlineStr">
         <is>
           <t>Mobile telecom, SIM cards, ISP broadband data tariffs.</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="G11" s="11" t="inlineStr">
         <is>
           <t>NIS Cambodia / CSES Household Survey</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="12" ht="40" customHeight="1">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>09</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Recreation and Culture</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C12" s="16" t="inlineStr">
         <is>
           <t>1.900%</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D12" s="16" t="inlineStr">
         <is>
           <t>Jevons Geometric Mean</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E12" s="16" t="inlineStr">
         <is>
           <t>Modified Laspeyres</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>Entertainment, electronics, leisure.</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>NIS Cambodia / CSES Household Survey</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="13" ht="40" customHeight="1">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>Education</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C13" s="17" t="inlineStr">
         <is>
           <t>1.500%</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D13" s="17" t="inlineStr">
         <is>
           <t>Jevons Geometric Mean</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E13" s="17" t="inlineStr">
         <is>
           <t>Modified Laspeyres</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F13" s="11" t="inlineStr">
         <is>
           <t>Tuition fees, textbooks, stationery.</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="G13" s="11" t="inlineStr">
         <is>
           <t>NIS Cambodia / CSES Household Survey</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="14" ht="40" customHeight="1">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Restaurants and Hotels</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C14" s="16" t="inlineStr">
         <is>
           <t>3.100%</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D14" s="16" t="inlineStr">
         <is>
           <t>Jevons Geometric Mean</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E14" s="16" t="inlineStr">
         <is>
           <t>Modified Laspeyres</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>Food away from home, street food vendors, hospitality.</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>NIS Cambodia / CSES Household Survey</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="15" ht="40" customHeight="1">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>Miscellaneous Goods and Services</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C15" s="17" t="inlineStr">
         <is>
           <t>2.200%</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D15" s="17" t="inlineStr">
         <is>
           <t>Jevons Geometric Mean</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E15" s="17" t="inlineStr">
         <is>
           <t>Modified Laspeyres</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F15" s="11" t="inlineStr">
         <is>
           <t>Personal care, financial services, FX fees.</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="G15" s="11" t="inlineStr">
         <is>
           <t>NIS Cambodia / CSES Household Survey</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="16" ht="40" customHeight="1">
+      <c r="A16" s="18" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B16" s="19" t="inlineStr">
         <is>
           <t>NATIONAL HEADLINE CPI BASKET</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C16" s="18" t="inlineStr">
         <is>
           <t>100.000%</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D16" s="18" t="inlineStr">
         <is>
           <t>Axiomatic Jevons</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E16" s="18" t="inlineStr">
         <is>
           <t>Modified Laspeyres</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F16" s="19" t="inlineStr">
         <is>
           <t>Headline CPI tracks complete national cost-of-living basket.</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="G16" s="19" t="inlineStr">
         <is>
           <t>Royal Government of Cambodia / MoP</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G14"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>